<commit_message>
Escape every value in the HTML report
CodeQL flagged report data being inserted into the page as HTML: status
codes, counts, response times and the category class name were not
escaped. Crawled values are numbers, but an edited or crafted JSON report
could inject markup. Also match the test's DNS-failure URL by hostname
instead of a prefix.
</commit_message>
<xml_diff>
--- a/docs/sample-report.xlsx
+++ b/docs/sample-report.xlsx
@@ -43,7 +43,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>10/19/2026, 6:24:11 PM</t>
+    <t>10/19/2026, 6:28:31 PM</t>
   </si>
   <si>
     <t>Duration (s)</t>
@@ -1027,7 +1027,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1421,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="V3">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="W3" t="s">
         <v>67</v>
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="V4">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="W4" t="s">
         <v>57</v>
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="V5">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="W5" t="s">
         <v>57</v>
@@ -1652,7 +1652,7 @@
         <v>2</v>
       </c>
       <c r="V6">
-        <v>93</v>
+        <v>181</v>
       </c>
       <c r="W6" t="s">
         <v>57</v>
@@ -1729,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="V7">
-        <v>71</v>
+        <v>295</v>
       </c>
       <c r="W7" t="s">
         <v>67</v>
@@ -1806,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="V8">
-        <v>83</v>
+        <v>355</v>
       </c>
       <c r="W8" t="s">
         <v>67</v>
@@ -1883,7 +1883,7 @@
         <v>2</v>
       </c>
       <c r="V9">
-        <v>17</v>
+        <v>249</v>
       </c>
       <c r="W9" t="s">
         <v>57</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="V10">
-        <v>18</v>
+        <v>217</v>
       </c>
       <c r="W10" t="s">
         <v>57</v>
@@ -2037,7 +2037,7 @@
         <v>1</v>
       </c>
       <c r="V11">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="W11" t="s">
         <v>57</v>
@@ -2114,7 +2114,7 @@
         <v>1</v>
       </c>
       <c r="V12">
-        <v>69</v>
+        <v>339</v>
       </c>
       <c r="W12" t="s">
         <v>57</v>
@@ -2191,7 +2191,7 @@
         <v>1</v>
       </c>
       <c r="V13">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="W13" t="s">
         <v>57</v>
@@ -2268,7 +2268,7 @@
         <v>1</v>
       </c>
       <c r="V14">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="W14" t="s">
         <v>57</v>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="V15">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="W15" t="s">
         <v>57</v>
@@ -2422,7 +2422,7 @@
         <v>1</v>
       </c>
       <c r="V16">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="W16" t="s">
         <v>57</v>
@@ -2499,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="V17">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="W17" t="s">
         <v>67</v>
@@ -2576,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="V18">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="W18" t="s">
         <v>67</v>
@@ -2653,7 +2653,7 @@
         <v>1</v>
       </c>
       <c r="V19">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W19" t="s">
         <v>57</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="V20">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="W20" t="s">
         <v>67</v>
@@ -2807,7 +2807,7 @@
         <v>1</v>
       </c>
       <c r="V21">
-        <v>112</v>
+        <v>388</v>
       </c>
       <c r="W21" t="s">
         <v>57</v>
@@ -2884,7 +2884,7 @@
         <v>2</v>
       </c>
       <c r="V22">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="W22" t="s">
         <v>57</v>
@@ -2961,7 +2961,7 @@
         <v>1</v>
       </c>
       <c r="V23">
-        <v>18</v>
+        <v>216</v>
       </c>
       <c r="W23" t="s">
         <v>57</v>
@@ -3038,7 +3038,7 @@
         <v>1</v>
       </c>
       <c r="V24">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="W24" t="s">
         <v>57</v>
@@ -3115,7 +3115,7 @@
         <v>1</v>
       </c>
       <c r="V25">
-        <v>18</v>
+        <v>251</v>
       </c>
       <c r="W25" t="s">
         <v>57</v>
@@ -3192,7 +3192,7 @@
         <v>1</v>
       </c>
       <c r="V26">
-        <v>97</v>
+        <v>369</v>
       </c>
       <c r="W26" t="s">
         <v>57</v>
@@ -3269,7 +3269,7 @@
         <v>2</v>
       </c>
       <c r="V27">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="W27" t="s">
         <v>57</v>
@@ -3346,7 +3346,7 @@
         <v>2</v>
       </c>
       <c r="V28">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="W28" t="s">
         <v>57</v>
@@ -3423,7 +3423,7 @@
         <v>3</v>
       </c>
       <c r="V29">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W29" t="s">
         <v>57</v>
@@ -3500,7 +3500,7 @@
         <v>3</v>
       </c>
       <c r="V30">
-        <v>2</v>
+        <v>523</v>
       </c>
       <c r="W30" t="s">
         <v>57</v>
@@ -3577,7 +3577,7 @@
         <v>2</v>
       </c>
       <c r="V31">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="W31" t="s">
         <v>57</v>
@@ -3654,7 +3654,7 @@
         <v>2</v>
       </c>
       <c r="V32">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="W32" t="s">
         <v>57</v>
@@ -3731,7 +3731,7 @@
         <v>1</v>
       </c>
       <c r="V33">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W33" t="s">
         <v>57</v>
@@ -3808,7 +3808,7 @@
         <v>1</v>
       </c>
       <c r="V34">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="W34" t="s">
         <v>57</v>
@@ -3885,7 +3885,7 @@
         <v>0</v>
       </c>
       <c r="V35">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="W35" t="s">
         <v>67</v>
@@ -4039,7 +4039,7 @@
         <v>1</v>
       </c>
       <c r="V37">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="W37" t="s">
         <v>57</v>
@@ -4116,7 +4116,7 @@
         <v>1</v>
       </c>
       <c r="V38">
-        <v>13</v>
+        <v>555</v>
       </c>
       <c r="W38" t="s">
         <v>57</v>
@@ -4193,7 +4193,7 @@
         <v>3</v>
       </c>
       <c r="V39">
-        <v>12</v>
+        <v>565</v>
       </c>
       <c r="W39" t="s">
         <v>57</v>
@@ -4270,7 +4270,7 @@
         <v>1</v>
       </c>
       <c r="V40">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="W40" t="s">
         <v>57</v>
@@ -4347,7 +4347,7 @@
         <v>1</v>
       </c>
       <c r="V41">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="W41" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Fix accessibility issues and update uuid
</commit_message>
<xml_diff>
--- a/docs/sample-report.xlsx
+++ b/docs/sample-report.xlsx
@@ -43,7 +43,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>10/19/2026, 6:28:31 PM</t>
+    <t>10/20/2026, 12:28:34 PM</t>
   </si>
   <si>
     <t>Duration (s)</t>
@@ -1027,7 +1027,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1421,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="V3">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="W3" t="s">
         <v>67</v>
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="V4">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="W4" t="s">
         <v>57</v>
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="V5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="W5" t="s">
         <v>57</v>
@@ -1652,7 +1652,7 @@
         <v>2</v>
       </c>
       <c r="V6">
-        <v>181</v>
+        <v>51</v>
       </c>
       <c r="W6" t="s">
         <v>57</v>
@@ -1729,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="V7">
-        <v>295</v>
+        <v>53</v>
       </c>
       <c r="W7" t="s">
         <v>67</v>
@@ -1806,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="V8">
-        <v>355</v>
+        <v>59</v>
       </c>
       <c r="W8" t="s">
         <v>67</v>
@@ -1883,7 +1883,7 @@
         <v>2</v>
       </c>
       <c r="V9">
-        <v>249</v>
+        <v>11</v>
       </c>
       <c r="W9" t="s">
         <v>57</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="V10">
-        <v>217</v>
+        <v>12</v>
       </c>
       <c r="W10" t="s">
         <v>57</v>
@@ -2037,7 +2037,7 @@
         <v>1</v>
       </c>
       <c r="V11">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="W11" t="s">
         <v>57</v>
@@ -2114,7 +2114,7 @@
         <v>1</v>
       </c>
       <c r="V12">
-        <v>339</v>
+        <v>48</v>
       </c>
       <c r="W12" t="s">
         <v>57</v>
@@ -2191,7 +2191,7 @@
         <v>1</v>
       </c>
       <c r="V13">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="W13" t="s">
         <v>57</v>
@@ -2268,7 +2268,7 @@
         <v>1</v>
       </c>
       <c r="V14">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="W14" t="s">
         <v>57</v>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="V15">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="W15" t="s">
         <v>57</v>
@@ -2422,7 +2422,7 @@
         <v>1</v>
       </c>
       <c r="V16">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="W16" t="s">
         <v>57</v>
@@ -2499,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="V17">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="W17" t="s">
         <v>67</v>
@@ -2576,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="V18">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="W18" t="s">
         <v>67</v>
@@ -2653,7 +2653,7 @@
         <v>1</v>
       </c>
       <c r="V19">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="W19" t="s">
         <v>57</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="V20">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="W20" t="s">
         <v>67</v>
@@ -2807,7 +2807,7 @@
         <v>1</v>
       </c>
       <c r="V21">
-        <v>388</v>
+        <v>69</v>
       </c>
       <c r="W21" t="s">
         <v>57</v>
@@ -2884,7 +2884,7 @@
         <v>2</v>
       </c>
       <c r="V22">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="W22" t="s">
         <v>57</v>
@@ -2961,7 +2961,7 @@
         <v>1</v>
       </c>
       <c r="V23">
-        <v>216</v>
+        <v>12</v>
       </c>
       <c r="W23" t="s">
         <v>57</v>
@@ -3038,7 +3038,7 @@
         <v>1</v>
       </c>
       <c r="V24">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="W24" t="s">
         <v>57</v>
@@ -3115,7 +3115,7 @@
         <v>1</v>
       </c>
       <c r="V25">
-        <v>251</v>
+        <v>13</v>
       </c>
       <c r="W25" t="s">
         <v>57</v>
@@ -3192,7 +3192,7 @@
         <v>1</v>
       </c>
       <c r="V26">
-        <v>369</v>
+        <v>62</v>
       </c>
       <c r="W26" t="s">
         <v>57</v>
@@ -3269,7 +3269,7 @@
         <v>2</v>
       </c>
       <c r="V27">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="W27" t="s">
         <v>57</v>
@@ -3346,7 +3346,7 @@
         <v>2</v>
       </c>
       <c r="V28">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="W28" t="s">
         <v>57</v>
@@ -3423,7 +3423,7 @@
         <v>3</v>
       </c>
       <c r="V29">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W29" t="s">
         <v>57</v>
@@ -3500,7 +3500,7 @@
         <v>3</v>
       </c>
       <c r="V30">
-        <v>523</v>
+        <v>2</v>
       </c>
       <c r="W30" t="s">
         <v>57</v>
@@ -3577,7 +3577,7 @@
         <v>2</v>
       </c>
       <c r="V31">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="W31" t="s">
         <v>57</v>
@@ -3654,7 +3654,7 @@
         <v>2</v>
       </c>
       <c r="V32">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="W32" t="s">
         <v>57</v>
@@ -3731,7 +3731,7 @@
         <v>1</v>
       </c>
       <c r="V33">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="W33" t="s">
         <v>57</v>
@@ -3808,7 +3808,7 @@
         <v>1</v>
       </c>
       <c r="V34">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="W34" t="s">
         <v>57</v>
@@ -3885,7 +3885,7 @@
         <v>0</v>
       </c>
       <c r="V35">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="W35" t="s">
         <v>67</v>
@@ -4039,7 +4039,7 @@
         <v>1</v>
       </c>
       <c r="V37">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="W37" t="s">
         <v>57</v>
@@ -4116,7 +4116,7 @@
         <v>1</v>
       </c>
       <c r="V38">
-        <v>555</v>
+        <v>7</v>
       </c>
       <c r="W38" t="s">
         <v>57</v>
@@ -4193,7 +4193,7 @@
         <v>3</v>
       </c>
       <c r="V39">
-        <v>565</v>
+        <v>5</v>
       </c>
       <c r="W39" t="s">
         <v>57</v>
@@ -4270,7 +4270,7 @@
         <v>1</v>
       </c>
       <c r="V40">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="W40" t="s">
         <v>57</v>
@@ -4347,7 +4347,7 @@
         <v>1</v>
       </c>
       <c r="V41">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="W41" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Fix accessibility issues and update uuid (#13)
Fixes colour contrast in the HTML report, landmarks and keyboard access
on the website, and forces uuid 11.1.1+ to clear the Dependabot alert.
</commit_message>
<xml_diff>
--- a/docs/sample-report.xlsx
+++ b/docs/sample-report.xlsx
@@ -43,7 +43,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>10/19/2026, 6:28:31 PM</t>
+    <t>10/20/2026, 12:28:34 PM</t>
   </si>
   <si>
     <t>Duration (s)</t>
@@ -1027,7 +1027,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1421,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="V3">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="W3" t="s">
         <v>67</v>
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="V4">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="W4" t="s">
         <v>57</v>
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="V5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="W5" t="s">
         <v>57</v>
@@ -1652,7 +1652,7 @@
         <v>2</v>
       </c>
       <c r="V6">
-        <v>181</v>
+        <v>51</v>
       </c>
       <c r="W6" t="s">
         <v>57</v>
@@ -1729,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="V7">
-        <v>295</v>
+        <v>53</v>
       </c>
       <c r="W7" t="s">
         <v>67</v>
@@ -1806,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="V8">
-        <v>355</v>
+        <v>59</v>
       </c>
       <c r="W8" t="s">
         <v>67</v>
@@ -1883,7 +1883,7 @@
         <v>2</v>
       </c>
       <c r="V9">
-        <v>249</v>
+        <v>11</v>
       </c>
       <c r="W9" t="s">
         <v>57</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="V10">
-        <v>217</v>
+        <v>12</v>
       </c>
       <c r="W10" t="s">
         <v>57</v>
@@ -2037,7 +2037,7 @@
         <v>1</v>
       </c>
       <c r="V11">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="W11" t="s">
         <v>57</v>
@@ -2114,7 +2114,7 @@
         <v>1</v>
       </c>
       <c r="V12">
-        <v>339</v>
+        <v>48</v>
       </c>
       <c r="W12" t="s">
         <v>57</v>
@@ -2191,7 +2191,7 @@
         <v>1</v>
       </c>
       <c r="V13">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="W13" t="s">
         <v>57</v>
@@ -2268,7 +2268,7 @@
         <v>1</v>
       </c>
       <c r="V14">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="W14" t="s">
         <v>57</v>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="V15">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="W15" t="s">
         <v>57</v>
@@ -2422,7 +2422,7 @@
         <v>1</v>
       </c>
       <c r="V16">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="W16" t="s">
         <v>57</v>
@@ -2499,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="V17">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="W17" t="s">
         <v>67</v>
@@ -2576,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="V18">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="W18" t="s">
         <v>67</v>
@@ -2653,7 +2653,7 @@
         <v>1</v>
       </c>
       <c r="V19">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="W19" t="s">
         <v>57</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="V20">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="W20" t="s">
         <v>67</v>
@@ -2807,7 +2807,7 @@
         <v>1</v>
       </c>
       <c r="V21">
-        <v>388</v>
+        <v>69</v>
       </c>
       <c r="W21" t="s">
         <v>57</v>
@@ -2884,7 +2884,7 @@
         <v>2</v>
       </c>
       <c r="V22">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="W22" t="s">
         <v>57</v>
@@ -2961,7 +2961,7 @@
         <v>1</v>
       </c>
       <c r="V23">
-        <v>216</v>
+        <v>12</v>
       </c>
       <c r="W23" t="s">
         <v>57</v>
@@ -3038,7 +3038,7 @@
         <v>1</v>
       </c>
       <c r="V24">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="W24" t="s">
         <v>57</v>
@@ -3115,7 +3115,7 @@
         <v>1</v>
       </c>
       <c r="V25">
-        <v>251</v>
+        <v>13</v>
       </c>
       <c r="W25" t="s">
         <v>57</v>
@@ -3192,7 +3192,7 @@
         <v>1</v>
       </c>
       <c r="V26">
-        <v>369</v>
+        <v>62</v>
       </c>
       <c r="W26" t="s">
         <v>57</v>
@@ -3269,7 +3269,7 @@
         <v>2</v>
       </c>
       <c r="V27">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="W27" t="s">
         <v>57</v>
@@ -3346,7 +3346,7 @@
         <v>2</v>
       </c>
       <c r="V28">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="W28" t="s">
         <v>57</v>
@@ -3423,7 +3423,7 @@
         <v>3</v>
       </c>
       <c r="V29">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W29" t="s">
         <v>57</v>
@@ -3500,7 +3500,7 @@
         <v>3</v>
       </c>
       <c r="V30">
-        <v>523</v>
+        <v>2</v>
       </c>
       <c r="W30" t="s">
         <v>57</v>
@@ -3577,7 +3577,7 @@
         <v>2</v>
       </c>
       <c r="V31">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="W31" t="s">
         <v>57</v>
@@ -3654,7 +3654,7 @@
         <v>2</v>
       </c>
       <c r="V32">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="W32" t="s">
         <v>57</v>
@@ -3731,7 +3731,7 @@
         <v>1</v>
       </c>
       <c r="V33">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="W33" t="s">
         <v>57</v>
@@ -3808,7 +3808,7 @@
         <v>1</v>
       </c>
       <c r="V34">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="W34" t="s">
         <v>57</v>
@@ -3885,7 +3885,7 @@
         <v>0</v>
       </c>
       <c r="V35">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="W35" t="s">
         <v>67</v>
@@ -4039,7 +4039,7 @@
         <v>1</v>
       </c>
       <c r="V37">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="W37" t="s">
         <v>57</v>
@@ -4116,7 +4116,7 @@
         <v>1</v>
       </c>
       <c r="V38">
-        <v>555</v>
+        <v>7</v>
       </c>
       <c r="W38" t="s">
         <v>57</v>
@@ -4193,7 +4193,7 @@
         <v>3</v>
       </c>
       <c r="V39">
-        <v>565</v>
+        <v>5</v>
       </c>
       <c r="W39" t="s">
         <v>57</v>
@@ -4270,7 +4270,7 @@
         <v>1</v>
       </c>
       <c r="V40">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="W40" t="s">
         <v>57</v>
@@ -4347,7 +4347,7 @@
         <v>1</v>
       </c>
       <c r="V41">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="W41" t="s">
         <v>57</v>

</xml_diff>